<commit_message>
updated more templates and fixed arrow size display on starting circles
</commit_message>
<xml_diff>
--- a/docs/seep/files/xslope_clay_blanket.xlsx
+++ b/docs/seep/files/xslope_clay_blanket.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/seep/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57438D71-D127-0142-BD65-3022A87A9D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06578632-4AD1-194D-8D67-0A6527FD7C96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="26660" yWindow="2680" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
@@ -1050,13 +1050,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1081,7 +1081,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -10170,37 +10191,37 @@
     <mergeCell ref="R7:V7"/>
   </mergeCells>
   <conditionalFormatting sqref="E9:F50">
-    <cfRule type="expression" dxfId="6" priority="4">
+    <cfRule type="expression" dxfId="9" priority="4">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:H50">
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="8" priority="3">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:J50">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M9:N50">
-    <cfRule type="expression" dxfId="3" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9:O50">
-    <cfRule type="expression" dxfId="2" priority="14">
+    <cfRule type="expression" dxfId="5" priority="14">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P9:Q50">
-    <cfRule type="expression" dxfId="1" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R9:V9">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10254,74 +10275,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="D4" s="47" t="s">
+      <c r="B4" s="45"/>
+      <c r="D4" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="G4" s="47" t="s">
+      <c r="E4" s="45"/>
+      <c r="G4" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="47"/>
-      <c r="J4" s="47" t="s">
+      <c r="H4" s="45"/>
+      <c r="J4" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="47"/>
-      <c r="M4" s="47" t="s">
+      <c r="K4" s="45"/>
+      <c r="M4" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="47"/>
-      <c r="P4" s="47" t="s">
+      <c r="N4" s="45"/>
+      <c r="P4" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="47"/>
+      <c r="Q4" s="45"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="47" t="s">
+      <c r="S4" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="47"/>
+      <c r="T4" s="45"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="47" t="s">
+      <c r="V4" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="47"/>
+      <c r="W4" s="45"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="47" t="s">
+      <c r="Y4" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="47"/>
+      <c r="Z4" s="45"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="47" t="s">
+      <c r="AB4" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="47"/>
-      <c r="AE4" s="47" t="s">
+      <c r="AC4" s="45"/>
+      <c r="AE4" s="45" t="s">
         <v>116</v>
       </c>
-      <c r="AF4" s="47"/>
+      <c r="AF4" s="45"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="47" t="s">
+      <c r="AH4" s="45" t="s">
         <v>117</v>
       </c>
-      <c r="AI4" s="47"/>
+      <c r="AI4" s="45"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="47" t="s">
+      <c r="AK4" s="45" t="s">
         <v>118</v>
       </c>
-      <c r="AL4" s="47"/>
+      <c r="AL4" s="45"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="47" t="s">
+      <c r="AN4" s="45" t="s">
         <v>119</v>
       </c>
-      <c r="AO4" s="47"/>
+      <c r="AO4" s="45"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="47" t="s">
+      <c r="AQ4" s="45" t="s">
         <v>120</v>
       </c>
-      <c r="AR4" s="47"/>
+      <c r="AR4" s="45"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -10424,89 +10445,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="45" t="str">
+      <c r="A6" s="46" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>soil</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="D6" s="45" t="str">
+      <c r="B6" s="47"/>
+      <c r="D6" s="46" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="46"/>
-      <c r="G6" s="45" t="str">
+      <c r="E6" s="47"/>
+      <c r="G6" s="46" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="46"/>
-      <c r="J6" s="45" t="str">
+      <c r="H6" s="47"/>
+      <c r="J6" s="46" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="46"/>
-      <c r="M6" s="45" t="str">
+      <c r="K6" s="47"/>
+      <c r="M6" s="46" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="46"/>
-      <c r="P6" s="45" t="str">
+      <c r="N6" s="47"/>
+      <c r="P6" s="46" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="46"/>
+      <c r="Q6" s="47"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="45" t="str">
+      <c r="S6" s="46" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="46"/>
+      <c r="T6" s="47"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="45" t="str">
+      <c r="V6" s="46" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="46"/>
+      <c r="W6" s="47"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="45" t="str">
+      <c r="Y6" s="46" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="46"/>
+      <c r="Z6" s="47"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="45" t="str">
+      <c r="AB6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="46"/>
-      <c r="AE6" s="45" t="str">
+      <c r="AC6" s="47"/>
+      <c r="AE6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="46"/>
+      <c r="AF6" s="47"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="45" t="str">
+      <c r="AH6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="46"/>
+      <c r="AI6" s="47"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="45" t="str">
+      <c r="AK6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="46"/>
+      <c r="AL6" s="47"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="45" t="str">
+      <c r="AN6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="46"/>
+      <c r="AO6" s="47"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="45" t="str">
+      <c r="AQ6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="46"/>
+      <c r="AR6" s="47"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -11434,36 +11455,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11821,12 +11842,24 @@
       <c r="N16" s="1"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D12" xr:uid="{06E9E004-FC39-FE49-926A-912F810F5089}">
+  <conditionalFormatting sqref="E3:E42">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>OR($D3="Intercept", $D3="Radius")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:G42">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>OR($D3="Depth",$D3="Radius")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H42">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>OR($D3="Depth",$D3="Intercept")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D52" xr:uid="{270ABC96-248F-0048-BDB9-DCF89EA62E14}">
       <formula1>$J$3:$J$5</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D4" xr:uid="{AEFC92A9-AB07-FF4B-9461-938B9BDCD07D}">
-      <formula1>$J$5:$J$7</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data+docs(seep): the clay-blanket file drops its unused unsat values
Owner's call: cells a confined problem never reads have no business
carrying numbers, and their explanation is SEEP-2's job. The sample's
kr0/h0/a/n cells are blank (round-tripped; the tag still reads 39.983),
both build paths dismiss everything after unsat in one sentence pointing
at SEEP-2, and the mat render and materials capture regenerate. Known
cosmetic asymmetry: the sheet is blank while Studio's editor shows the
loader-coerced zeros.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/seep/files/xslope_clay_blanket.xlsx
+++ b/docs/seep/files/xslope_clay_blanket.xlsx
@@ -6657,18 +6657,10 @@
           <t>lf</t>
         </is>
       </c>
-      <c r="AK11" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="AL11" s="3">
-        <v>-1.0</v>
-      </c>
-      <c r="AM11" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="AN11" s="3">
-        <v>0.0</v>
-      </c>
+      <c r="AK11" s="3"/>
+      <c r="AL11" s="3"/>
+      <c r="AM11" s="3"/>
+      <c r="AN11" s="3"/>
       <c r="AO11" s="3"/>
       <c r="AP11" s="3"/>
     </row>

</xml_diff>

<commit_message>
data+docs(seep): the unsat selector goes blank with its parameters
The owner meant all of them: a blank unsat cell loads as lf by default, so
the sheet now carries nothing across the whole unsaturated tail, the page
says so, and the Studio step notes the editor shows the lf default for the
blank cell. Tag still 39.983.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/seep/files/xslope_clay_blanket.xlsx
+++ b/docs/seep/files/xslope_clay_blanket.xlsx
@@ -6652,15 +6652,19 @@
       <c r="AI11" s="3">
         <v>0.0</v>
       </c>
-      <c r="AJ11" s="3" t="inlineStr">
-        <is>
-          <t>lf</t>
-        </is>
-      </c>
-      <c r="AK11" s="3"/>
-      <c r="AL11" s="3"/>
-      <c r="AM11" s="3"/>
-      <c r="AN11" s="3"/>
+      <c r="AJ11" s="3"/>
+      <c r="AK11" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="AL11" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="AM11" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="AN11" s="3">
+        <v>0.0</v>
+      </c>
       <c r="AO11" s="3"/>
       <c r="AP11" s="3"/>
     </row>

</xml_diff>